<commit_message>
Corrige columnas_llave en DIM_SATELITE_DEF a nombres de columna legibles por el motor
Antes: descripcion verbose con alias y corchetes de tipo
Ahora: solo expresiones minimas - COALESCE(per_ncode,ins_ncode), aco_ncode, cit_ncode

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CcS2rRicqWu6BQakKjvAJK
</commit_message>
<xml_diff>
--- a/pruebas/CA003_Plantilla_parametrizacion_e_ingesta_de_reglas_SPRINT_2_vs3.xlsx
+++ b/pruebas/CA003_Plantilla_parametrizacion_e_ingesta_de_reglas_SPRINT_2_vs3.xlsx
@@ -2045,7 +2045,7 @@
     <col width="12.15234375" bestFit="1" customWidth="1" style="114" min="11" max="11"/>
     <col width="15.23046875" customWidth="1" style="114" min="12" max="12"/>
     <col width="7.3046875" customWidth="1" style="114" min="13" max="14"/>
-    <col hidden="1" style="114" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" style="114" min="15" max="15"/>
     <col hidden="1" width="7.3046875" customWidth="1" style="114" min="16" max="17"/>
     <col hidden="1" width="7.3046875" customWidth="1" style="114" min="18" max="16384"/>
   </cols>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="D5" s="125" t="inlineStr">
         <is>
-          <t>Columnas de union entre tablas, separadas por punto y coma. Incluye el tipo de union (ENTIDAD / COMUN / COMPUESTA) y las tablas implicadas.</t>
+          <t>Columnas de union entre tablas. Una por linea. Para llaves simples: nombre_columna. Para llaves derivadas: expresion SQL minima, ej. COALESCE(col_a, col_b). Para llaves compuestas: substr(col1),col2 o col1,col2.</t>
         </is>
       </c>
       <c r="E5" s="125" t="inlineStr">
@@ -3267,11 +3267,9 @@
       </c>
       <c r="D6" s="126" t="inlineStr">
         <is>
-          <t xml:space="preserve">base → addr    : COALESCE(PER_NCODE, INS_NCODE) = COALESCE(PER_NCODE, INS_NCODE)  [ENTIDAD]
-base → aco     : COALESCE(PER_NCODE, INS_NCODE) = COALESCE(PER_NCODE, INS_NCODE)  [ENTIDAD]
-aco  → mem     : ACO_NCODE = ACO_NCODE  (auto-detectada como *_NCODE comun)         [COMUN]
-addr → ciu     : CIT_NCODE = CIT_NCODE  (auto-detectada como *_NCODE comun)         [COMUN]
-</t>
+          <t>COALESCE(per_ncode, ins_ncode)
+aco_ncode
+cit_ncode</t>
         </is>
       </c>
       <c r="E6" s="126" t="inlineStr">

</xml_diff>